<commit_message>
finding tauc exceedance in spring events!!!!!
</commit_message>
<xml_diff>
--- a/correlations/hysteresis_bed_conc.xlsx
+++ b/correlations/hysteresis_bed_conc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\hysteresis\correlations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6076C902-4A04-4DA6-BF0B-8B736616E903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A37944F2-7EE6-4B73-B5F5-B05CDBEF7AD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{867610DC-2157-4A8B-BAD4-C3624B9432BC}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="32">
   <si>
     <t>Storm</t>
   </si>
@@ -131,6 +131,74 @@
   <si>
     <t>Peak concentration (mg/L)</t>
   </si>
+  <si>
+    <r>
+      <t>Time between events (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>τ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>c exceedance)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (hrs)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Time between events (no </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>τ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>c exceedance)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (hrs)</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -143,7 +211,7 @@
     <numFmt numFmtId="167" formatCode="0.0000"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -158,6 +226,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -3031,8 +3112,8 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.27466743914535768"/>
-          <c:y val="0.17171296296296298"/>
+          <c:x val="0.2568302039168181"/>
+          <c:y val="0.24115740740740746"/>
           <c:w val="0.67302486854694998"/>
           <c:h val="0.51718321668124823"/>
         </c:manualLayout>
@@ -8091,7 +8172,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.276072296982944"/>
+          <c:y val="0.24115740740740746"/>
+          <c:w val="0.59973595273834923"/>
+          <c:h val="0.60106408573928261"/>
+        </c:manualLayout>
+      </c:layout>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
@@ -8907,6 +8998,733 @@
       </c:legendEntry>
       <c:legendEntry>
         <c:idx val="5"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart19.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" baseline="0"/>
+              <a:t>Bed POC to time between storms (no </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="el-GR" sz="1200" baseline="0"/>
+              <a:t>τ</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" baseline="0"/>
+              <a:t>c exceedance)</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="1200"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.31498534626852187"/>
+          <c:y val="0.17430555555555555"/>
+          <c:w val="0.56914888360589089"/>
+          <c:h val="0.45729841061533977"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'V1 '!$F$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Reach Bed POC (mgC/mg)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="0"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="0.15913627687929166"/>
+                  <c:y val="-6.1175998833479191E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="20000"/>
+                    <a:lumOff val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'V1 '!$F$6:$F$10</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>1.7629051004676988E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.3683478327705962E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.8181317207464335E-2</c:v>
+                </c:pt>
+                <c:pt idx="3" formatCode="0.0000">
+                  <c:v>3.0644232792768952E-2</c:v>
+                </c:pt>
+                <c:pt idx="4" formatCode="0.0000">
+                  <c:v>5.0676335550048197E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'V1 '!$I$6:$I$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>118.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2036.95</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2036.95</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>365</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>365</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-4BEB-4B22-9D9B-17250FBF6F7F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'V1 '!$G$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Average Bed POC (mgC/mg)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="0"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="0.23173542250180701"/>
+                  <c:y val="-0.1912153689122193"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="20000"/>
+                    <a:lumOff val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'V1 '!$G$6:$G$10</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>2.3018230827484512E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.0932397767585145E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.0932397767585145E-2</c:v>
+                </c:pt>
+                <c:pt idx="3" formatCode="0.0000">
+                  <c:v>4.0660284171408573E-2</c:v>
+                </c:pt>
+                <c:pt idx="4" formatCode="0.0000">
+                  <c:v>4.0660284171408573E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'V1 '!$I$6:$I$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>118.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2036.95</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2036.95</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>365</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>365</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-4BEB-4B22-9D9B-17250FBF6F7F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1602320480"/>
+        <c:axId val="1602307040"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1602320480"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Bed POC (mgC/mg)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00000" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1602307040"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1602307040"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Peak </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> concentration (mg/L)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.000" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1602320480"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:legendEntry>
+        <c:idx val="2"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:legendEntry>
+        <c:idx val="3"/>
         <c:delete val="1"/>
       </c:legendEntry>
       <c:overlay val="0"/>
@@ -16842,6 +17660,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors19.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -22322,6 +23180,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style19.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -26687,13 +28061,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>405493</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>46944</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>253093</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>65994</xdr:rowOff>
@@ -26723,13 +28097,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>329293</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>51707</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>910318</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>70757</xdr:rowOff>
@@ -26761,13 +28135,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>405493</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>127907</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>253093</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>13607</xdr:rowOff>
@@ -26799,13 +28173,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>357868</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>132670</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>938893</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>18370</xdr:rowOff>
@@ -26837,13 +28211,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>405493</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>51707</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>253093</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>127907</xdr:rowOff>
@@ -26875,13 +28249,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>357868</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>56470</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>938893</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>132670</xdr:rowOff>
@@ -26913,13 +28287,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>107977</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>39941</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>302960</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>58991</xdr:rowOff>
@@ -26951,13 +28325,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>138793</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>127907</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>333776</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>13607</xdr:rowOff>
@@ -26989,13 +28363,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>148318</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>42182</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>343301</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>118382</xdr:rowOff>
@@ -27027,13 +28401,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>1000125</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
+      <xdr:col>21</xdr:col>
       <xdr:colOff>161925</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
@@ -27065,13 +28439,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>971550</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
+      <xdr:col>21</xdr:col>
       <xdr:colOff>133350</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>9525</xdr:rowOff>
@@ -27103,16 +28477,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>1000125</xdr:colOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>962025</xdr:colOff>
       <xdr:row>28</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>161925</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
       <xdr:row>41</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -27134,6 +28508,44 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>238125</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>23533</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="10" name="Chart 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{888C2186-D213-4034-BA3E-92A7F020EC79}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -28996,7 +30408,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24B27869-60E0-43BF-B7FC-18286E7E1076}">
-  <dimension ref="A1:Q53"/>
+  <dimension ref="A1:R53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" style="1" customWidth="1"/>
@@ -29005,17 +30417,17 @@
     <col min="5" max="5" width="18.7109375" customWidth="1"/>
     <col min="6" max="6" width="19.7109375" customWidth="1"/>
     <col min="7" max="7" width="18.140625" customWidth="1"/>
-    <col min="8" max="8" width="22.28515625" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" customWidth="1"/>
-    <col min="10" max="10" width="21.42578125" customWidth="1"/>
-    <col min="11" max="12" width="16" customWidth="1"/>
-    <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="16.28515625" customWidth="1"/>
-    <col min="15" max="15" width="17.7109375" customWidth="1"/>
-    <col min="16" max="16" width="18.7109375" customWidth="1"/>
+    <col min="8" max="9" width="22.28515625" customWidth="1"/>
+    <col min="10" max="10" width="18.140625" customWidth="1"/>
+    <col min="11" max="11" width="21.42578125" customWidth="1"/>
+    <col min="12" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="13" customWidth="1"/>
+    <col min="15" max="15" width="16.28515625" customWidth="1"/>
+    <col min="16" max="16" width="17.7109375" customWidth="1"/>
+    <col min="17" max="17" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B1" s="10" t="s">
         <v>12</v>
       </c>
@@ -29023,21 +30435,21 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
-      <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="1"/>
+      <c r="O1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
     </row>
-    <row r="2" spans="1:17" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="12" t="s">
         <v>0</v>
       </c>
@@ -29059,15 +30471,18 @@
       <c r="H2" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="I2" s="14"/>
-      <c r="K2" s="1"/>
+      <c r="I2" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="J2" s="14"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
-      <c r="O2" s="1"/>
+      <c r="N2" s="1"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
@@ -29089,15 +30504,16 @@
       <c r="H3" s="16">
         <v>562.32579999999996</v>
       </c>
-      <c r="I3" s="3"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="3"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="3"/>
+      <c r="L3" s="1"/>
       <c r="M3" s="3"/>
-      <c r="O3" s="1"/>
+      <c r="N3" s="3"/>
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
+      <c r="R3" s="1"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
@@ -29119,15 +30535,16 @@
       <c r="H4" s="16">
         <v>359.22</v>
       </c>
-      <c r="K4" s="1"/>
-      <c r="L4" s="3"/>
+      <c r="I4" s="1"/>
+      <c r="L4" s="1"/>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
-      <c r="O4" s="1"/>
+      <c r="O4" s="3"/>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>4</v>
       </c>
@@ -29149,15 +30566,18 @@
       <c r="H5" s="16">
         <v>57.726100000000002</v>
       </c>
-      <c r="K5" s="1"/>
-      <c r="L5" s="3"/>
+      <c r="I5" s="1">
+        <v>9023.75</v>
+      </c>
+      <c r="L5" s="1"/>
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
-      <c r="O5" s="9"/>
-      <c r="P5" s="1"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="9"/>
       <c r="Q5" s="1"/>
+      <c r="R5" s="1"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>5</v>
       </c>
@@ -29179,15 +30599,18 @@
       <c r="H6" s="16">
         <v>49.091801670000002</v>
       </c>
-      <c r="K6" s="1"/>
-      <c r="L6" s="3"/>
+      <c r="I6" s="1">
+        <v>118.5</v>
+      </c>
+      <c r="L6" s="1"/>
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="1"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="9"/>
       <c r="Q6" s="1"/>
+      <c r="R6" s="1"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>25</v>
       </c>
@@ -29212,15 +30635,18 @@
       <c r="H7" s="16">
         <v>187</v>
       </c>
-      <c r="K7" s="1"/>
-      <c r="L7" s="3"/>
+      <c r="I7" s="1">
+        <v>2036.95</v>
+      </c>
+      <c r="L7" s="1"/>
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="1"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="9"/>
       <c r="Q7" s="1"/>
+      <c r="R7" s="1"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>7</v>
       </c>
@@ -29242,15 +30668,18 @@
       <c r="H8" s="16">
         <v>105.55555560000001</v>
       </c>
-      <c r="K8" s="1"/>
-      <c r="L8" s="3"/>
+      <c r="I8" s="1">
+        <v>2036.95</v>
+      </c>
+      <c r="L8" s="1"/>
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="1"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="9"/>
       <c r="Q8" s="1"/>
+      <c r="R8" s="1"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
@@ -29266,15 +30695,18 @@
       <c r="H9" s="16">
         <v>76.153846150000007</v>
       </c>
-      <c r="K9" s="1"/>
-      <c r="L9" s="3"/>
+      <c r="I9" s="1">
+        <v>365</v>
+      </c>
+      <c r="L9" s="1"/>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="1"/>
+      <c r="O9" s="3"/>
+      <c r="P9" s="9"/>
       <c r="Q9" s="1"/>
+      <c r="R9" s="1"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>25</v>
       </c>
@@ -29299,17 +30731,20 @@
       <c r="H10" s="16">
         <v>43.2</v>
       </c>
-      <c r="I10" s="9"/>
-      <c r="J10" s="1"/>
+      <c r="I10" s="1">
+        <v>365</v>
+      </c>
+      <c r="J10" s="9"/>
       <c r="K10" s="1"/>
-      <c r="L10" s="3"/>
+      <c r="L10" s="1"/>
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
-      <c r="O10" s="9"/>
-      <c r="P10" s="1"/>
+      <c r="O10" s="3"/>
+      <c r="P10" s="9"/>
       <c r="Q10" s="1"/>
+      <c r="R10" s="1"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
         <v>9</v>
       </c>
@@ -29326,15 +30761,18 @@
       <c r="H11" s="16">
         <v>77.894736839999993</v>
       </c>
-      <c r="K11" s="1"/>
-      <c r="L11" s="3"/>
+      <c r="I11" s="1">
+        <v>351.5</v>
+      </c>
+      <c r="L11" s="1"/>
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
-      <c r="O11" s="9"/>
-      <c r="P11" s="1"/>
+      <c r="O11" s="3"/>
+      <c r="P11" s="9"/>
       <c r="Q11" s="1"/>
+      <c r="R11" s="1"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>10</v>
       </c>
@@ -29352,15 +30790,18 @@
       <c r="H12" s="16">
         <v>37.6</v>
       </c>
-      <c r="K12" s="1"/>
+      <c r="I12" s="1">
+        <v>413.75</v>
+      </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
-      <c r="N12" s="11"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="11"/>
+      <c r="P12" s="9"/>
       <c r="Q12" s="1"/>
+      <c r="R12" s="1"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>11</v>
       </c>
@@ -29378,15 +30819,18 @@
       <c r="H13" s="16">
         <v>30.76923077</v>
       </c>
-      <c r="K13" s="1"/>
+      <c r="I13" s="1">
+        <v>413.75</v>
+      </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="9"/>
-      <c r="P13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="11"/>
+      <c r="P13" s="9"/>
       <c r="Q13" s="1"/>
+      <c r="R13" s="1"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -29395,7 +30839,7 @@
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
       <c r="I14" s="9"/>
-      <c r="J14" s="1"/>
+      <c r="J14" s="9"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
@@ -29403,8 +30847,9 @@
       <c r="O14" s="1"/>
       <c r="P14" s="1"/>
       <c r="Q14" s="1"/>
+      <c r="R14" s="1"/>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B15" s="10" t="s">
         <v>14</v>
       </c>
@@ -29423,8 +30868,9 @@
       <c r="O15" s="1"/>
       <c r="P15" s="1"/>
       <c r="Q15" s="1"/>
+      <c r="R15" s="1"/>
     </row>
-    <row r="16" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="B16" s="12" t="s">
         <v>0</v>
       </c>
@@ -29446,8 +30892,10 @@
       <c r="H16" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="I16" s="14"/>
-      <c r="J16" s="1"/>
+      <c r="I16" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="J16" s="14"/>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
@@ -29455,8 +30903,9 @@
       <c r="O16" s="1"/>
       <c r="P16" s="1"/>
       <c r="Q16" s="1"/>
+      <c r="R16" s="1"/>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
         <v>2</v>
       </c>
@@ -29478,16 +30927,17 @@
       <c r="H17" s="16">
         <v>13.39</v>
       </c>
-      <c r="J17" s="1"/>
+      <c r="I17" s="16"/>
       <c r="K17" s="1"/>
-      <c r="L17" s="3"/>
+      <c r="L17" s="1"/>
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
-      <c r="O17" s="1"/>
+      <c r="O17" s="3"/>
       <c r="P17" s="1"/>
       <c r="Q17" s="1"/>
+      <c r="R17" s="1"/>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
         <v>3</v>
       </c>
@@ -29509,16 +30959,17 @@
       <c r="H18" s="16">
         <v>13.108000000000001</v>
       </c>
-      <c r="J18" s="1"/>
+      <c r="I18" s="1"/>
       <c r="K18" s="1"/>
-      <c r="L18" s="3"/>
+      <c r="L18" s="1"/>
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
-      <c r="O18" s="1"/>
+      <c r="O18" s="3"/>
       <c r="P18" s="1"/>
       <c r="Q18" s="1"/>
+      <c r="R18" s="1"/>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
         <v>4</v>
       </c>
@@ -29540,16 +30991,19 @@
       <c r="H19" s="16">
         <v>8.6910000000000007</v>
       </c>
-      <c r="J19" s="1"/>
+      <c r="I19" s="1">
+        <v>9023.75</v>
+      </c>
       <c r="K19" s="1"/>
-      <c r="L19" s="3"/>
+      <c r="L19" s="1"/>
       <c r="M19" s="3"/>
       <c r="N19" s="3"/>
-      <c r="O19" s="9"/>
-      <c r="P19" s="1"/>
+      <c r="O19" s="3"/>
+      <c r="P19" s="9"/>
       <c r="Q19" s="1"/>
+      <c r="R19" s="1"/>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>5</v>
       </c>
@@ -29571,16 +31025,19 @@
       <c r="H20" s="16">
         <v>8.4209999999999994</v>
       </c>
-      <c r="J20" s="1"/>
+      <c r="I20" s="1">
+        <v>118.5</v>
+      </c>
       <c r="K20" s="1"/>
-      <c r="L20" s="3"/>
+      <c r="L20" s="1"/>
       <c r="M20" s="3"/>
       <c r="N20" s="3"/>
-      <c r="O20" s="9"/>
-      <c r="P20" s="1"/>
+      <c r="O20" s="3"/>
+      <c r="P20" s="9"/>
       <c r="Q20" s="1"/>
+      <c r="R20" s="1"/>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>25</v>
       </c>
@@ -29605,16 +31062,19 @@
       <c r="H21" s="16">
         <v>5.15</v>
       </c>
-      <c r="J21" s="1"/>
+      <c r="I21" s="1">
+        <v>2036.95</v>
+      </c>
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
-      <c r="O21" s="9"/>
-      <c r="P21" s="1"/>
+      <c r="O21" s="1"/>
+      <c r="P21" s="9"/>
       <c r="Q21" s="1"/>
+      <c r="R21" s="1"/>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>7</v>
       </c>
@@ -29636,16 +31096,19 @@
       <c r="H22" s="16">
         <v>8.5760000000000005</v>
       </c>
-      <c r="J22" s="1"/>
+      <c r="I22" s="1">
+        <v>2036.95</v>
+      </c>
       <c r="K22" s="1"/>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
       <c r="N22" s="1"/>
-      <c r="O22" s="9"/>
-      <c r="P22" s="1"/>
+      <c r="O22" s="1"/>
+      <c r="P22" s="9"/>
       <c r="Q22" s="1"/>
+      <c r="R22" s="1"/>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>17</v>
       </c>
@@ -29661,16 +31124,19 @@
       <c r="H23" s="16">
         <v>4.4729999999999999</v>
       </c>
-      <c r="J23" s="1"/>
+      <c r="I23" s="1">
+        <v>365</v>
+      </c>
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
-      <c r="O23" s="9"/>
-      <c r="P23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="9"/>
       <c r="Q23" s="1"/>
+      <c r="R23" s="1"/>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>25</v>
       </c>
@@ -29695,16 +31161,19 @@
       <c r="H24" s="16">
         <v>9.9</v>
       </c>
-      <c r="J24" s="1"/>
+      <c r="I24" s="1">
+        <v>365</v>
+      </c>
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
-      <c r="O24" s="9"/>
-      <c r="P24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="9"/>
       <c r="Q24" s="1"/>
+      <c r="R24" s="1"/>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>25</v>
       </c>
@@ -29725,16 +31194,19 @@
       <c r="H25" s="16">
         <v>4.2779999999999996</v>
       </c>
-      <c r="J25" s="1"/>
+      <c r="I25" s="1">
+        <v>351.5</v>
+      </c>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
       <c r="N25" s="1"/>
-      <c r="O25" s="9"/>
-      <c r="P25" s="1"/>
+      <c r="O25" s="1"/>
+      <c r="P25" s="9"/>
       <c r="Q25" s="1"/>
+      <c r="R25" s="1"/>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
         <v>10</v>
       </c>
@@ -29751,15 +31223,18 @@
       <c r="H26" s="16">
         <v>5.4009999999999998</v>
       </c>
-      <c r="K26" s="1"/>
+      <c r="I26" s="1">
+        <v>413.75</v>
+      </c>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
       <c r="N26" s="1"/>
-      <c r="O26" s="9"/>
-      <c r="P26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="9"/>
       <c r="Q26" s="1"/>
+      <c r="R26" s="1"/>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
         <v>11</v>
       </c>
@@ -29776,22 +31251,24 @@
       <c r="H27" s="16">
         <v>8.7050000000000001</v>
       </c>
-      <c r="J27" s="1"/>
+      <c r="I27" s="1">
+        <v>413.75</v>
+      </c>
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
       <c r="N27" s="1"/>
-      <c r="O27" s="9"/>
-      <c r="P27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="9"/>
       <c r="Q27" s="1"/>
+      <c r="R27" s="1"/>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B28" s="1"/>
       <c r="C28" s="2"/>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
-      <c r="J28" s="1"/>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -29799,8 +31276,9 @@
       <c r="O28" s="1"/>
       <c r="P28" s="1"/>
       <c r="Q28" s="1"/>
+      <c r="R28" s="1"/>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B29" s="10" t="s">
         <v>13</v>
       </c>
@@ -29819,8 +31297,9 @@
       <c r="O29" s="1"/>
       <c r="P29" s="1"/>
       <c r="Q29" s="1"/>
+      <c r="R29" s="1"/>
     </row>
-    <row r="30" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="B30" s="12" t="s">
         <v>0</v>
       </c>
@@ -29842,8 +31321,10 @@
       <c r="H30" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="I30" s="14"/>
-      <c r="J30" s="1"/>
+      <c r="I30" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="J30" s="14"/>
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -29851,8 +31332,9 @@
       <c r="O30" s="1"/>
       <c r="P30" s="1"/>
       <c r="Q30" s="1"/>
+      <c r="R30" s="1"/>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
         <v>2</v>
       </c>
@@ -29874,17 +31356,18 @@
       <c r="H31" s="15">
         <v>51.66</v>
       </c>
-      <c r="I31" s="3"/>
-      <c r="J31" s="1"/>
+      <c r="I31" s="16"/>
+      <c r="J31" s="3"/>
       <c r="K31" s="1"/>
-      <c r="L31" s="3"/>
+      <c r="L31" s="1"/>
       <c r="M31" s="3"/>
       <c r="N31" s="3"/>
-      <c r="O31" s="1"/>
+      <c r="O31" s="3"/>
       <c r="P31" s="1"/>
       <c r="Q31" s="1"/>
+      <c r="R31" s="1"/>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B32" s="1" t="s">
         <v>3</v>
       </c>
@@ -29906,17 +31389,18 @@
       <c r="H32" s="15">
         <v>41.27935076</v>
       </c>
-      <c r="I32" s="3"/>
-      <c r="J32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="3"/>
       <c r="K32" s="1"/>
-      <c r="L32" s="3"/>
+      <c r="L32" s="1"/>
       <c r="M32" s="3"/>
       <c r="N32" s="3"/>
-      <c r="O32" s="1"/>
+      <c r="O32" s="3"/>
       <c r="P32" s="1"/>
       <c r="Q32" s="1"/>
+      <c r="R32" s="1"/>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
         <v>4</v>
       </c>
@@ -29938,17 +31422,20 @@
       <c r="H33" s="15">
         <v>6.7843516800000003</v>
       </c>
-      <c r="I33" s="3"/>
-      <c r="J33" s="1"/>
+      <c r="I33" s="1">
+        <v>9023.75</v>
+      </c>
+      <c r="J33" s="3"/>
       <c r="K33" s="1"/>
-      <c r="L33" s="3"/>
+      <c r="L33" s="1"/>
       <c r="M33" s="3"/>
       <c r="N33" s="3"/>
-      <c r="O33" s="9"/>
-      <c r="P33" s="1"/>
+      <c r="O33" s="3"/>
+      <c r="P33" s="9"/>
       <c r="Q33" s="1"/>
+      <c r="R33" s="1"/>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B34" s="1" t="s">
         <v>5</v>
       </c>
@@ -29970,16 +31457,19 @@
       <c r="H34" s="15">
         <v>5.3650916630000003</v>
       </c>
-      <c r="I34" s="3"/>
-      <c r="K34" s="1"/>
-      <c r="L34" s="3"/>
+      <c r="I34" s="1">
+        <v>118.5</v>
+      </c>
+      <c r="J34" s="3"/>
+      <c r="L34" s="1"/>
       <c r="M34" s="3"/>
       <c r="N34" s="3"/>
-      <c r="O34" s="9"/>
-      <c r="P34" s="1"/>
+      <c r="O34" s="3"/>
+      <c r="P34" s="9"/>
       <c r="Q34" s="1"/>
+      <c r="R34" s="1"/>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>25</v>
       </c>
@@ -30004,17 +31494,20 @@
       <c r="H35" s="15">
         <v>29.943162610000002</v>
       </c>
-      <c r="I35" s="3"/>
-      <c r="J35" s="1"/>
+      <c r="I35" s="1">
+        <v>2036.95</v>
+      </c>
+      <c r="J35" s="3"/>
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
       <c r="N35" s="1"/>
-      <c r="O35" s="9"/>
-      <c r="P35" s="1"/>
+      <c r="O35" s="1"/>
+      <c r="P35" s="9"/>
       <c r="Q35" s="1"/>
+      <c r="R35" s="1"/>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B36" s="1" t="s">
         <v>7</v>
       </c>
@@ -30036,17 +31529,20 @@
       <c r="H36" s="15">
         <v>13.904999999999999</v>
       </c>
-      <c r="I36" s="3"/>
-      <c r="J36" s="1"/>
+      <c r="I36" s="1">
+        <v>2036.95</v>
+      </c>
+      <c r="J36" s="3"/>
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
       <c r="N36" s="1"/>
-      <c r="O36" s="9"/>
-      <c r="P36" s="1"/>
+      <c r="O36" s="1"/>
+      <c r="P36" s="9"/>
       <c r="Q36" s="1"/>
+      <c r="R36" s="1"/>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
         <v>17</v>
       </c>
@@ -30062,17 +31558,20 @@
       <c r="H37" s="15">
         <v>7.7779999999999996</v>
       </c>
-      <c r="I37" s="9"/>
-      <c r="J37" s="1"/>
+      <c r="I37" s="1">
+        <v>365</v>
+      </c>
+      <c r="J37" s="9"/>
       <c r="K37" s="1"/>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
       <c r="N37" s="1"/>
-      <c r="O37" s="9"/>
-      <c r="P37" s="1"/>
+      <c r="O37" s="1"/>
+      <c r="P37" s="9"/>
       <c r="Q37" s="1"/>
+      <c r="R37" s="1"/>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>25</v>
       </c>
@@ -30097,17 +31596,20 @@
       <c r="H38" s="15">
         <v>5.5549999999999997</v>
       </c>
-      <c r="I38" s="9"/>
-      <c r="J38" s="1"/>
+      <c r="I38" s="1">
+        <v>365</v>
+      </c>
+      <c r="J38" s="9"/>
       <c r="K38" s="1"/>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
       <c r="N38" s="1"/>
-      <c r="O38" s="9"/>
-      <c r="P38" s="1"/>
+      <c r="O38" s="1"/>
+      <c r="P38" s="9"/>
       <c r="Q38" s="1"/>
+      <c r="R38" s="1"/>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B39" s="1" t="s">
         <v>9</v>
       </c>
@@ -30125,17 +31627,20 @@
       <c r="H39" s="15">
         <v>12.67</v>
       </c>
-      <c r="I39" s="9"/>
-      <c r="J39" s="1"/>
+      <c r="I39" s="1">
+        <v>351.5</v>
+      </c>
+      <c r="J39" s="9"/>
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
       <c r="N39" s="1"/>
-      <c r="O39" s="9"/>
-      <c r="P39" s="1"/>
+      <c r="O39" s="1"/>
+      <c r="P39" s="9"/>
       <c r="Q39" s="1"/>
+      <c r="R39" s="1"/>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
         <v>10</v>
       </c>
@@ -30153,17 +31658,20 @@
       <c r="H40" s="15">
         <v>5.3390000000000004</v>
       </c>
-      <c r="I40" s="9"/>
-      <c r="J40" s="1"/>
+      <c r="I40" s="1">
+        <v>413.75</v>
+      </c>
+      <c r="J40" s="9"/>
       <c r="K40" s="1"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
       <c r="N40" s="1"/>
-      <c r="O40" s="9"/>
-      <c r="P40" s="1"/>
+      <c r="O40" s="1"/>
+      <c r="P40" s="9"/>
       <c r="Q40" s="1"/>
+      <c r="R40" s="1"/>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B41" s="1" t="s">
         <v>11</v>
       </c>
@@ -30181,17 +31689,20 @@
       <c r="H41" s="15">
         <v>5.1369999999999996</v>
       </c>
-      <c r="I41" s="9"/>
-      <c r="J41" s="1"/>
+      <c r="I41" s="1">
+        <v>413.75</v>
+      </c>
+      <c r="J41" s="9"/>
       <c r="K41" s="1"/>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
       <c r="N41" s="1"/>
-      <c r="O41" s="9"/>
-      <c r="P41" s="1"/>
+      <c r="O41" s="1"/>
+      <c r="P41" s="9"/>
       <c r="Q41" s="1"/>
+      <c r="R41" s="1"/>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
@@ -30208,8 +31719,9 @@
       <c r="O42" s="1"/>
       <c r="P42" s="1"/>
       <c r="Q42" s="1"/>
+      <c r="R42" s="1"/>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B43" s="1" t="s">
         <v>19</v>
       </c>
@@ -30230,27 +31742,28 @@
       </c>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
-      <c r="K43" s="1" t="s">
+      <c r="J43" s="1"/>
+      <c r="L43" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="L43" s="1" t="s">
+      <c r="M43" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="M43" s="1" t="s">
+      <c r="N43" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="N43" s="1" t="s">
+      <c r="O43" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="O43" s="1" t="s">
+      <c r="P43" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="P43" s="1" t="s">
+      <c r="Q43" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q43" s="1"/>
+      <c r="R43" s="1"/>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B44" s="1" t="s">
         <v>2</v>
       </c>
@@ -30271,27 +31784,28 @@
       </c>
       <c r="H44" s="3"/>
       <c r="I44" s="3"/>
-      <c r="K44" s="1" t="s">
+      <c r="J44" s="3"/>
+      <c r="L44" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="L44" s="8">
+      <c r="M44" s="8">
         <v>0.46925034971041901</v>
       </c>
-      <c r="M44" s="8">
+      <c r="N44" s="8">
         <v>-0.57047580585715596</v>
       </c>
-      <c r="N44" s="8">
+      <c r="O44" s="8">
         <v>-0.62489073949006502</v>
       </c>
-      <c r="O44" s="8">
+      <c r="P44" s="8">
         <v>-0.505884156285488</v>
       </c>
-      <c r="P44" s="8">
+      <c r="Q44" s="8">
         <v>-0.62313135244567197</v>
       </c>
-      <c r="Q44" s="1"/>
+      <c r="R44" s="1"/>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B45" s="1" t="s">
         <v>3</v>
       </c>
@@ -30312,27 +31826,28 @@
       </c>
       <c r="H45" s="3"/>
       <c r="I45" s="3"/>
-      <c r="K45" s="1" t="s">
+      <c r="J45" s="3"/>
+      <c r="L45" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="L45" s="8">
+      <c r="M45" s="8">
         <v>0.52770506265369399</v>
       </c>
-      <c r="M45" s="8">
+      <c r="N45" s="8">
         <v>-0.57441925876348399</v>
       </c>
-      <c r="N45" s="8">
+      <c r="O45" s="8">
         <v>-0.61127875482433702</v>
       </c>
-      <c r="O45" s="8">
+      <c r="P45" s="8">
         <v>-0.50988466103239405</v>
       </c>
-      <c r="P45" s="8">
+      <c r="Q45" s="8">
         <v>-0.59410954788831905</v>
       </c>
-      <c r="Q45" s="1"/>
+      <c r="R45" s="1"/>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B46" s="1" t="s">
         <v>4</v>
       </c>
@@ -30353,28 +31868,29 @@
       </c>
       <c r="H46" s="3"/>
       <c r="I46" s="3"/>
-      <c r="J46" s="9"/>
-      <c r="K46" s="1" t="s">
+      <c r="J46" s="3"/>
+      <c r="K46" s="9"/>
+      <c r="L46" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="L46" s="8">
+      <c r="M46" s="8">
         <v>0.76151296818251002</v>
       </c>
-      <c r="M46" s="8">
+      <c r="N46" s="8">
         <v>-0.82455849900808098</v>
       </c>
-      <c r="N46" s="8">
+      <c r="O46" s="8">
         <v>-0.53010922957415696</v>
       </c>
-      <c r="O46" s="8">
+      <c r="P46" s="8">
         <v>-0.67807302432253402</v>
       </c>
-      <c r="P46" s="8">
+      <c r="Q46" s="8">
         <v>-0.81917889363282403</v>
       </c>
-      <c r="Q46" s="1"/>
+      <c r="R46" s="1"/>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B47" s="1" t="s">
         <v>5</v>
       </c>
@@ -30395,28 +31911,29 @@
       </c>
       <c r="H47" s="3"/>
       <c r="I47" s="3"/>
-      <c r="J47" s="9"/>
-      <c r="K47" s="1" t="s">
+      <c r="J47" s="3"/>
+      <c r="K47" s="9"/>
+      <c r="L47" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="L47" s="8">
+      <c r="M47" s="8">
         <v>0.63241662033349</v>
       </c>
-      <c r="M47" s="8">
+      <c r="N47" s="8">
         <v>-0.77305412456000899</v>
       </c>
-      <c r="N47" s="8">
+      <c r="O47" s="8">
         <v>-0.511670862423525</v>
       </c>
-      <c r="O47" s="8">
+      <c r="P47" s="8">
         <v>-0.62213976025652196</v>
       </c>
-      <c r="P47" s="8">
+      <c r="Q47" s="8">
         <v>-0.76662036881149098</v>
       </c>
-      <c r="Q47" s="1"/>
+      <c r="R47" s="1"/>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B48" s="1" t="s">
         <v>6</v>
       </c>
@@ -30437,28 +31954,29 @@
       </c>
       <c r="H48" s="3"/>
       <c r="I48" s="3"/>
-      <c r="J48" s="9"/>
-      <c r="K48" s="1" t="s">
+      <c r="J48" s="3"/>
+      <c r="K48" s="9"/>
+      <c r="L48" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="L48" s="8">
+      <c r="M48" s="8">
         <v>0.68587815994758305</v>
       </c>
-      <c r="M48" s="8">
+      <c r="N48" s="8">
         <v>-0.74314055155585101</v>
       </c>
-      <c r="N48" s="8">
+      <c r="O48" s="8">
         <v>-0.22155858359451899</v>
       </c>
-      <c r="O48" s="8">
+      <c r="P48" s="8">
         <v>-0.51680913320449795</v>
       </c>
-      <c r="P48" s="8">
+      <c r="Q48" s="8">
         <v>-0.79093223163479298</v>
       </c>
-      <c r="Q48" s="1"/>
+      <c r="R48" s="1"/>
     </row>
-    <row r="49" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B49" s="1" t="s">
         <v>7</v>
       </c>
@@ -30479,28 +31997,29 @@
       </c>
       <c r="H49" s="3"/>
       <c r="I49" s="3"/>
-      <c r="J49" s="9"/>
-      <c r="K49" s="1" t="s">
+      <c r="J49" s="3"/>
+      <c r="K49" s="9"/>
+      <c r="L49" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="L49" s="8">
+      <c r="M49" s="8">
         <v>0.64478493475432996</v>
       </c>
-      <c r="M49" s="8">
+      <c r="N49" s="8">
         <v>-0.64445784381595494</v>
       </c>
-      <c r="N49" s="8">
+      <c r="O49" s="8">
         <v>-0.24334139198969101</v>
       </c>
-      <c r="O49" s="8">
+      <c r="P49" s="8">
         <v>-0.34407999236201098</v>
       </c>
-      <c r="P49" s="8">
+      <c r="Q49" s="8">
         <v>-0.52379920048275397</v>
       </c>
-      <c r="Q49" s="1"/>
+      <c r="R49" s="1"/>
     </row>
-    <row r="50" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B50" s="1" t="s">
         <v>17</v>
       </c>
@@ -30521,27 +32040,28 @@
       </c>
       <c r="H50" s="3"/>
       <c r="I50" s="3"/>
-      <c r="K50" s="1" t="s">
+      <c r="J50" s="3"/>
+      <c r="L50" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="L50" s="7">
+      <c r="M50" s="7">
         <v>1.04151195285145</v>
       </c>
-      <c r="M50" s="8">
+      <c r="N50" s="8">
         <v>-0.120988015114778</v>
       </c>
-      <c r="N50" s="7">
+      <c r="O50" s="7">
         <v>9.6450074853088597E-2</v>
       </c>
-      <c r="O50" s="8">
+      <c r="P50" s="8">
         <v>-5.48657708396144E-2</v>
       </c>
-      <c r="P50" s="8">
+      <c r="Q50" s="8">
         <v>-0.16320255139754999</v>
       </c>
-      <c r="Q50" s="1"/>
+      <c r="R50" s="1"/>
     </row>
-    <row r="51" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B51" s="1" t="s">
         <v>18</v>
       </c>
@@ -30562,27 +32082,28 @@
       </c>
       <c r="H51" s="3"/>
       <c r="I51" s="3"/>
-      <c r="K51" s="1" t="s">
+      <c r="J51" s="3"/>
+      <c r="L51" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="L51" s="8">
+      <c r="M51" s="8">
         <v>0.57916197400143898</v>
       </c>
-      <c r="M51" s="8">
+      <c r="N51" s="8">
         <v>-0.78477741945709301</v>
       </c>
-      <c r="N51" s="8">
+      <c r="O51" s="8">
         <v>-0.24313716774511701</v>
       </c>
-      <c r="O51" s="8">
+      <c r="P51" s="8">
         <v>-0.62437814022779903</v>
       </c>
-      <c r="P51" s="8">
+      <c r="Q51" s="8">
         <v>-0.748656600612842</v>
       </c>
-      <c r="Q51" s="1"/>
+      <c r="R51" s="1"/>
     </row>
-    <row r="52" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B52" s="1" t="s">
         <v>11</v>
       </c>
@@ -30603,28 +32124,29 @@
       </c>
       <c r="H52" s="3"/>
       <c r="I52" s="3"/>
-      <c r="J52" s="9"/>
-      <c r="K52" s="1" t="s">
+      <c r="J52" s="3"/>
+      <c r="K52" s="9"/>
+      <c r="L52" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="L52" s="8">
+      <c r="M52" s="8">
         <v>0.74506131022172795</v>
       </c>
-      <c r="M52" s="8">
+      <c r="N52" s="8">
         <v>-0.75894808346496501</v>
       </c>
-      <c r="N52" s="8">
+      <c r="O52" s="8">
         <v>-0.37958282657101999</v>
       </c>
-      <c r="O52" s="8">
+      <c r="P52" s="8">
         <v>-0.37092334927613402</v>
       </c>
-      <c r="P52" s="8">
+      <c r="Q52" s="8">
         <v>-0.49092006249230202</v>
       </c>
-      <c r="Q52" s="1"/>
+      <c r="R52" s="1"/>
     </row>
-    <row r="53" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
       <c r="D53" s="1"/>
@@ -30641,6 +32163,7 @@
       <c r="O53" s="1"/>
       <c r="P53" s="1"/>
       <c r="Q53" s="1"/>
+      <c r="R53" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
correlating bed POC concentration to time between tauc exceedance events
</commit_message>
<xml_diff>
--- a/correlations/hysteresis_bed_conc.xlsx
+++ b/correlations/hysteresis_bed_conc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\hysteresis\correlations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A37944F2-7EE6-4B73-B5F5-B05CDBEF7AD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9053F51B-E732-44D2-91CE-D2F550509CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{867610DC-2157-4A8B-BAD4-C3624B9432BC}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="32">
   <si>
     <t>Storm</t>
   </si>
@@ -132,12 +132,16 @@
     <t>Peak concentration (mg/L)</t>
   </si>
   <si>
+    <t>Time between events τc exceedance (hrs)</t>
+  </si>
+  <si>
     <r>
-      <t>Time between events (</t>
+      <t xml:space="preserve">Time between events (no </t>
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
+        <b/>
+        <sz val="10"/>
         <color theme="1"/>
         <rFont val="Aptos"/>
         <family val="2"/>
@@ -147,7 +151,8 @@
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
+        <b/>
+        <sz val="10"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
         <family val="2"/>
@@ -156,41 +161,8 @@
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (hrs)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Time between events (no </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t>τ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-      </rPr>
-      <t>c exceedance)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
+        <b/>
+        <sz val="10"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
         <family val="2"/>
@@ -211,7 +183,7 @@
     <numFmt numFmtId="167" formatCode="0.0000"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -228,14 +200,24 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Aptos"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -282,7 +264,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -331,6 +313,15 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9260,23 +9251,26 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'V1 '!$F$6:$F$10</c:f>
+              <c:f>'V1 '!$F$5:$F$10</c:f>
               <c:numCache>
                 <c:formatCode>0.00000</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>3.6863794196113527E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1.7629051004676988E-2</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>3.3683478327705962E-2</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2.8181317207464335E-2</c:v>
                 </c:pt>
-                <c:pt idx="3" formatCode="0.0000">
+                <c:pt idx="4" formatCode="0.0000">
                   <c:v>3.0644232792768952E-2</c:v>
                 </c:pt>
-                <c:pt idx="4" formatCode="0.0000">
+                <c:pt idx="5" formatCode="0.0000">
                   <c:v>5.0676335550048197E-2</c:v>
                 </c:pt>
               </c:numCache>
@@ -9284,23 +9278,26 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'V1 '!$I$6:$I$10</c:f>
+              <c:f>'V1 '!$I$5:$I$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>9023.75</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>118.5</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2036.95</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2036.95</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>2036.95</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>365</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>365</c:v>
                 </c:pt>
               </c:numCache>
@@ -9365,8 +9362,8 @@
             <c:trendlineLbl>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="0.23173542250180701"/>
-                  <c:y val="-0.1912153689122193"/>
+                  <c:x val="0.28080919840604984"/>
+                  <c:y val="-0.28395656379778861"/>
                 </c:manualLayout>
               </c:layout>
               <c:numFmt formatCode="General" sourceLinked="0"/>
@@ -9406,23 +9403,26 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'V1 '!$G$6:$G$10</c:f>
+              <c:f>'V1 '!$G$5:$G$10</c:f>
               <c:numCache>
                 <c:formatCode>0.00000</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>2.6974532065504243E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2.3018230827484512E-2</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>3.0932397767585145E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>3.0932397767585145E-2</c:v>
                 </c:pt>
-                <c:pt idx="3" formatCode="0.0000">
+                <c:pt idx="3">
+                  <c:v>3.0932397767585145E-2</c:v>
+                </c:pt>
+                <c:pt idx="4" formatCode="0.0000">
                   <c:v>4.0660284171408573E-2</c:v>
                 </c:pt>
-                <c:pt idx="4" formatCode="0.0000">
+                <c:pt idx="5" formatCode="0.0000">
                   <c:v>4.0660284171408573E-2</c:v>
                 </c:pt>
               </c:numCache>
@@ -9430,23 +9430,26 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'V1 '!$I$6:$I$10</c:f>
+              <c:f>'V1 '!$I$5:$I$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>9023.75</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>118.5</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2036.95</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2036.95</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>2036.95</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>365</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>365</c:v>
                 </c:pt>
               </c:numCache>
@@ -10683,6 +10686,721 @@
       </c:legendEntry>
       <c:legendEntry>
         <c:idx val="5"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart20.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" baseline="0"/>
+              <a:t>Bed POC to time between </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="el-GR" sz="1200" baseline="0"/>
+              <a:t>τ</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" baseline="0"/>
+              <a:t>c exceedance storms </a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="1200"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.31498534626852187"/>
+          <c:y val="0.17430555555555555"/>
+          <c:w val="0.56914888360589089"/>
+          <c:h val="0.45729841061533977"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'V1 '!$F$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Reach Bed POC (mgC/mg)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="0"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.21488436133985947"/>
+                  <c:y val="1.0513490524831607E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="20000"/>
+                    <a:lumOff val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'V1 '!$F$5:$F$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>3.6863794196113527E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.7629051004676988E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.3683478327705962E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.8181317207464335E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'V1 '!$J$5:$J$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>9023.75</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>118.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2060.9499999999998</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2060.9499999999998</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-5A65-4C15-A2B3-787A8CEE8EAB}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'V1 '!$G$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Average Bed POC (mgC/mg)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="0"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.12602743575288505"/>
+                  <c:y val="-0.19947899619008211"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="20000"/>
+                    <a:lumOff val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'V1 '!$G$5:$G$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2.6974532065504243E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.3018230827484512E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.0932397767585145E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.0932397767585145E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'V1 '!$J$5:$J$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>9023.75</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>118.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2060.9499999999998</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2060.9499999999998</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-5A65-4C15-A2B3-787A8CEE8EAB}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1602320480"/>
+        <c:axId val="1602307040"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1602320480"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Bed POC (mgC/mg)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00000" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1602307040"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1602307040"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Peak </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> concentration (mg/L)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.000" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1602320480"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:legendEntry>
+        <c:idx val="2"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:legendEntry>
+        <c:idx val="3"/>
         <c:delete val="1"/>
       </c:legendEntry>
       <c:overlay val="0"/>
@@ -17740,6 +18458,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors20.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -24212,6 +24970,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style20.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -28061,13 +29335,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>405493</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>46944</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>253093</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>65994</xdr:rowOff>
@@ -28097,13 +29371,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>329293</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>51707</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>910318</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>70757</xdr:rowOff>
@@ -28135,13 +29409,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>405493</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>127907</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>253093</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>13607</xdr:rowOff>
@@ -28173,13 +29447,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>357868</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>132670</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>938893</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>18370</xdr:rowOff>
@@ -28211,13 +29485,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>405493</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>51707</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>253093</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>127907</xdr:rowOff>
@@ -28249,13 +29523,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>357868</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>56470</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>938893</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>132670</xdr:rowOff>
@@ -28287,13 +29561,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>107977</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>39941</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>302960</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>58991</xdr:rowOff>
@@ -28325,13 +29599,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>138793</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>127907</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>333776</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>13607</xdr:rowOff>
@@ -28363,13 +29637,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>148318</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>42182</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>343301</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>118382</xdr:rowOff>
@@ -28401,13 +29675,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>1000125</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
+      <xdr:col>22</xdr:col>
       <xdr:colOff>161925</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
@@ -28439,13 +29713,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>971550</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
+      <xdr:col>22</xdr:col>
       <xdr:colOff>133350</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>9525</xdr:rowOff>
@@ -28477,13 +29751,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>962025</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
+      <xdr:col>22</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
@@ -28515,16 +29789,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>238125</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>306160</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>65314</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>23533</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>186818</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>138793</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -28546,6 +29820,44 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>244928</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>40820</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>397729</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>114299</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="9" name="Chart 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{871CBDCC-CC47-44BD-BB66-6C88DE56C2A1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -30408,7 +31720,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24B27869-60E0-43BF-B7FC-18286E7E1076}">
-  <dimension ref="A1:R53"/>
+  <dimension ref="A1:S53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" style="1" customWidth="1"/>
@@ -30417,17 +31729,17 @@
     <col min="5" max="5" width="18.7109375" customWidth="1"/>
     <col min="6" max="6" width="19.7109375" customWidth="1"/>
     <col min="7" max="7" width="18.140625" customWidth="1"/>
-    <col min="8" max="9" width="22.28515625" customWidth="1"/>
-    <col min="10" max="10" width="18.140625" customWidth="1"/>
-    <col min="11" max="11" width="21.42578125" customWidth="1"/>
-    <col min="12" max="13" width="16" customWidth="1"/>
-    <col min="14" max="14" width="13" customWidth="1"/>
-    <col min="15" max="15" width="16.28515625" customWidth="1"/>
-    <col min="16" max="16" width="17.7109375" customWidth="1"/>
-    <col min="17" max="17" width="18.7109375" customWidth="1"/>
+    <col min="8" max="10" width="22.28515625" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" customWidth="1"/>
+    <col min="12" max="12" width="21.42578125" customWidth="1"/>
+    <col min="13" max="14" width="16" customWidth="1"/>
+    <col min="15" max="15" width="13" customWidth="1"/>
+    <col min="16" max="16" width="16.28515625" customWidth="1"/>
+    <col min="17" max="17" width="17.7109375" customWidth="1"/>
+    <col min="18" max="18" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B1" s="10" t="s">
         <v>12</v>
       </c>
@@ -30435,54 +31747,57 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
-      <c r="L1" s="1"/>
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
-      <c r="O1" s="5" t="s">
+      <c r="O1" s="1"/>
+      <c r="P1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="Q1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="R1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
     </row>
-    <row r="2" spans="1:18" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="12" t="s">
+    <row r="2" spans="1:19" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="H2" s="14" t="s">
+      <c r="H2" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="I2" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="J2" s="14"/>
-      <c r="L2" s="1"/>
+      <c r="J2" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="K2" s="14"/>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
-      <c r="P2" s="1"/>
+      <c r="O2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
@@ -30505,15 +31820,16 @@
         <v>562.32579999999996</v>
       </c>
       <c r="I3" s="16"/>
-      <c r="J3" s="3"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="3"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="3"/>
+      <c r="M3" s="1"/>
       <c r="N3" s="3"/>
-      <c r="P3" s="1"/>
+      <c r="O3" s="3"/>
       <c r="Q3" s="1"/>
       <c r="R3" s="1"/>
+      <c r="S3" s="1"/>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
@@ -30536,15 +31852,16 @@
         <v>359.22</v>
       </c>
       <c r="I4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="3"/>
+      <c r="J4" s="1"/>
+      <c r="M4" s="1"/>
       <c r="N4" s="3"/>
       <c r="O4" s="3"/>
-      <c r="P4" s="1"/>
+      <c r="P4" s="3"/>
       <c r="Q4" s="1"/>
       <c r="R4" s="1"/>
+      <c r="S4" s="1"/>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>4</v>
       </c>
@@ -30569,15 +31886,18 @@
       <c r="I5" s="1">
         <v>9023.75</v>
       </c>
-      <c r="L5" s="1"/>
-      <c r="M5" s="3"/>
+      <c r="J5" s="1">
+        <v>9023.75</v>
+      </c>
+      <c r="M5" s="1"/>
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
-      <c r="P5" s="9"/>
-      <c r="Q5" s="1"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="9"/>
       <c r="R5" s="1"/>
+      <c r="S5" s="1"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>5</v>
       </c>
@@ -30602,15 +31922,18 @@
       <c r="I6" s="1">
         <v>118.5</v>
       </c>
-      <c r="L6" s="1"/>
-      <c r="M6" s="3"/>
+      <c r="J6" s="1">
+        <v>118.5</v>
+      </c>
+      <c r="M6" s="1"/>
       <c r="N6" s="3"/>
       <c r="O6" s="3"/>
-      <c r="P6" s="9"/>
-      <c r="Q6" s="1"/>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="9"/>
       <c r="R6" s="1"/>
+      <c r="S6" s="1"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>25</v>
       </c>
@@ -30638,15 +31961,18 @@
       <c r="I7" s="1">
         <v>2036.95</v>
       </c>
-      <c r="L7" s="1"/>
-      <c r="M7" s="3"/>
+      <c r="J7" s="1">
+        <v>2060.9499999999998</v>
+      </c>
+      <c r="M7" s="1"/>
       <c r="N7" s="3"/>
       <c r="O7" s="3"/>
-      <c r="P7" s="9"/>
-      <c r="Q7" s="1"/>
+      <c r="P7" s="3"/>
+      <c r="Q7" s="9"/>
       <c r="R7" s="1"/>
+      <c r="S7" s="1"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>7</v>
       </c>
@@ -30671,15 +31997,18 @@
       <c r="I8" s="1">
         <v>2036.95</v>
       </c>
-      <c r="L8" s="1"/>
-      <c r="M8" s="3"/>
+      <c r="J8" s="1">
+        <v>2060.9499999999998</v>
+      </c>
+      <c r="M8" s="1"/>
       <c r="N8" s="3"/>
       <c r="O8" s="3"/>
-      <c r="P8" s="9"/>
-      <c r="Q8" s="1"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="9"/>
       <c r="R8" s="1"/>
+      <c r="S8" s="1"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
@@ -30698,15 +32027,16 @@
       <c r="I9" s="1">
         <v>365</v>
       </c>
-      <c r="L9" s="1"/>
-      <c r="M9" s="3"/>
+      <c r="J9" s="1"/>
+      <c r="M9" s="1"/>
       <c r="N9" s="3"/>
       <c r="O9" s="3"/>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="1"/>
+      <c r="P9" s="3"/>
+      <c r="Q9" s="9"/>
       <c r="R9" s="1"/>
+      <c r="S9" s="1"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>25</v>
       </c>
@@ -30734,17 +32064,18 @@
       <c r="I10" s="1">
         <v>365</v>
       </c>
-      <c r="J10" s="9"/>
-      <c r="K10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="9"/>
       <c r="L10" s="1"/>
-      <c r="M10" s="3"/>
+      <c r="M10" s="1"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
-      <c r="P10" s="9"/>
-      <c r="Q10" s="1"/>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="9"/>
       <c r="R10" s="1"/>
+      <c r="S10" s="1"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
         <v>9</v>
       </c>
@@ -30764,15 +32095,16 @@
       <c r="I11" s="1">
         <v>351.5</v>
       </c>
-      <c r="L11" s="1"/>
-      <c r="M11" s="3"/>
+      <c r="J11" s="1"/>
+      <c r="M11" s="1"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
-      <c r="P11" s="9"/>
-      <c r="Q11" s="1"/>
+      <c r="P11" s="3"/>
+      <c r="Q11" s="9"/>
       <c r="R11" s="1"/>
+      <c r="S11" s="1"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>10</v>
       </c>
@@ -30793,15 +32125,18 @@
       <c r="I12" s="1">
         <v>413.75</v>
       </c>
-      <c r="L12" s="1"/>
+      <c r="J12" s="1">
+        <v>1130.25</v>
+      </c>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
-      <c r="O12" s="11"/>
-      <c r="P12" s="9"/>
-      <c r="Q12" s="1"/>
+      <c r="O12" s="1"/>
+      <c r="P12" s="11"/>
+      <c r="Q12" s="9"/>
       <c r="R12" s="1"/>
+      <c r="S12" s="1"/>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>11</v>
       </c>
@@ -30822,15 +32157,18 @@
       <c r="I13" s="1">
         <v>413.75</v>
       </c>
-      <c r="L13" s="1"/>
+      <c r="J13" s="1">
+        <v>1130.25</v>
+      </c>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
-      <c r="O13" s="11"/>
-      <c r="P13" s="9"/>
-      <c r="Q13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="11"/>
+      <c r="Q13" s="9"/>
       <c r="R13" s="1"/>
+      <c r="S13" s="1"/>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -30840,7 +32178,7 @@
       <c r="H14" s="9"/>
       <c r="I14" s="9"/>
       <c r="J14" s="9"/>
-      <c r="K14" s="1"/>
+      <c r="K14" s="9"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
@@ -30848,8 +32186,9 @@
       <c r="P14" s="1"/>
       <c r="Q14" s="1"/>
       <c r="R14" s="1"/>
+      <c r="S14" s="1"/>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B15" s="10" t="s">
         <v>14</v>
       </c>
@@ -30869,34 +32208,33 @@
       <c r="P15" s="1"/>
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
+      <c r="S15" s="1"/>
     </row>
-    <row r="16" spans="1:18" ht="30" x14ac:dyDescent="0.25">
-      <c r="B16" s="12" t="s">
+    <row r="16" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="B16" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="E16" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="F16" s="13" t="s">
+      <c r="F16" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="G16" s="13" t="s">
+      <c r="G16" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="H16" s="14" t="s">
+      <c r="H16" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I16" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="J16" s="14"/>
-      <c r="K16" s="1"/>
+      <c r="I16" s="18"/>
+      <c r="J16" s="18"/>
+      <c r="K16" s="14"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
@@ -30904,8 +32242,9 @@
       <c r="P16" s="1"/>
       <c r="Q16" s="1"/>
       <c r="R16" s="1"/>
+      <c r="S16" s="1"/>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
         <v>2</v>
       </c>
@@ -30928,16 +32267,17 @@
         <v>13.39</v>
       </c>
       <c r="I17" s="16"/>
-      <c r="K17" s="1"/>
+      <c r="J17" s="16"/>
       <c r="L17" s="1"/>
-      <c r="M17" s="3"/>
+      <c r="M17" s="1"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
-      <c r="P17" s="1"/>
+      <c r="P17" s="3"/>
       <c r="Q17" s="1"/>
       <c r="R17" s="1"/>
+      <c r="S17" s="1"/>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
         <v>3</v>
       </c>
@@ -30960,16 +32300,17 @@
         <v>13.108000000000001</v>
       </c>
       <c r="I18" s="1"/>
-      <c r="K18" s="1"/>
+      <c r="J18" s="1"/>
       <c r="L18" s="1"/>
-      <c r="M18" s="3"/>
+      <c r="M18" s="1"/>
       <c r="N18" s="3"/>
       <c r="O18" s="3"/>
-      <c r="P18" s="1"/>
+      <c r="P18" s="3"/>
       <c r="Q18" s="1"/>
       <c r="R18" s="1"/>
+      <c r="S18" s="1"/>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
         <v>4</v>
       </c>
@@ -30991,19 +32332,18 @@
       <c r="H19" s="16">
         <v>8.6910000000000007</v>
       </c>
-      <c r="I19" s="1">
-        <v>9023.75</v>
-      </c>
-      <c r="K19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
       <c r="L19" s="1"/>
-      <c r="M19" s="3"/>
+      <c r="M19" s="1"/>
       <c r="N19" s="3"/>
       <c r="O19" s="3"/>
-      <c r="P19" s="9"/>
-      <c r="Q19" s="1"/>
+      <c r="P19" s="3"/>
+      <c r="Q19" s="9"/>
       <c r="R19" s="1"/>
+      <c r="S19" s="1"/>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>5</v>
       </c>
@@ -31025,19 +32365,18 @@
       <c r="H20" s="16">
         <v>8.4209999999999994</v>
       </c>
-      <c r="I20" s="1">
-        <v>118.5</v>
-      </c>
-      <c r="K20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
       <c r="L20" s="1"/>
-      <c r="M20" s="3"/>
+      <c r="M20" s="1"/>
       <c r="N20" s="3"/>
       <c r="O20" s="3"/>
-      <c r="P20" s="9"/>
-      <c r="Q20" s="1"/>
+      <c r="P20" s="3"/>
+      <c r="Q20" s="9"/>
       <c r="R20" s="1"/>
+      <c r="S20" s="1"/>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>25</v>
       </c>
@@ -31062,19 +32401,18 @@
       <c r="H21" s="16">
         <v>5.15</v>
       </c>
-      <c r="I21" s="1">
-        <v>2036.95</v>
-      </c>
-      <c r="K21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
-      <c r="P21" s="9"/>
-      <c r="Q21" s="1"/>
+      <c r="P21" s="1"/>
+      <c r="Q21" s="9"/>
       <c r="R21" s="1"/>
+      <c r="S21" s="1"/>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>7</v>
       </c>
@@ -31096,19 +32434,18 @@
       <c r="H22" s="16">
         <v>8.5760000000000005</v>
       </c>
-      <c r="I22" s="1">
-        <v>2036.95</v>
-      </c>
-      <c r="K22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
-      <c r="P22" s="9"/>
-      <c r="Q22" s="1"/>
+      <c r="P22" s="1"/>
+      <c r="Q22" s="9"/>
       <c r="R22" s="1"/>
+      <c r="S22" s="1"/>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>17</v>
       </c>
@@ -31124,19 +32461,18 @@
       <c r="H23" s="16">
         <v>4.4729999999999999</v>
       </c>
-      <c r="I23" s="1">
-        <v>365</v>
-      </c>
-      <c r="K23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
-      <c r="P23" s="9"/>
-      <c r="Q23" s="1"/>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="9"/>
       <c r="R23" s="1"/>
+      <c r="S23" s="1"/>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>25</v>
       </c>
@@ -31161,19 +32497,18 @@
       <c r="H24" s="16">
         <v>9.9</v>
       </c>
-      <c r="I24" s="1">
-        <v>365</v>
-      </c>
-      <c r="K24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
       <c r="O24" s="1"/>
-      <c r="P24" s="9"/>
-      <c r="Q24" s="1"/>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="9"/>
       <c r="R24" s="1"/>
+      <c r="S24" s="1"/>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>25</v>
       </c>
@@ -31194,19 +32529,18 @@
       <c r="H25" s="16">
         <v>4.2779999999999996</v>
       </c>
-      <c r="I25" s="1">
-        <v>351.5</v>
-      </c>
-      <c r="K25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
       <c r="N25" s="1"/>
       <c r="O25" s="1"/>
-      <c r="P25" s="9"/>
-      <c r="Q25" s="1"/>
+      <c r="P25" s="1"/>
+      <c r="Q25" s="9"/>
       <c r="R25" s="1"/>
+      <c r="S25" s="1"/>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
         <v>10</v>
       </c>
@@ -31223,18 +32557,17 @@
       <c r="H26" s="16">
         <v>5.4009999999999998</v>
       </c>
-      <c r="I26" s="1">
-        <v>413.75</v>
-      </c>
-      <c r="L26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
       <c r="M26" s="1"/>
       <c r="N26" s="1"/>
       <c r="O26" s="1"/>
-      <c r="P26" s="9"/>
-      <c r="Q26" s="1"/>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="9"/>
       <c r="R26" s="1"/>
+      <c r="S26" s="1"/>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
         <v>11</v>
       </c>
@@ -31251,25 +32584,23 @@
       <c r="H27" s="16">
         <v>8.7050000000000001</v>
       </c>
-      <c r="I27" s="1">
-        <v>413.75</v>
-      </c>
-      <c r="K27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
       <c r="N27" s="1"/>
       <c r="O27" s="1"/>
-      <c r="P27" s="9"/>
-      <c r="Q27" s="1"/>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="9"/>
       <c r="R27" s="1"/>
+      <c r="S27" s="1"/>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B28" s="1"/>
       <c r="C28" s="2"/>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
-      <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
       <c r="N28" s="1"/>
@@ -31277,8 +32608,9 @@
       <c r="P28" s="1"/>
       <c r="Q28" s="1"/>
       <c r="R28" s="1"/>
+      <c r="S28" s="1"/>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B29" s="10" t="s">
         <v>13</v>
       </c>
@@ -31298,34 +32630,33 @@
       <c r="P29" s="1"/>
       <c r="Q29" s="1"/>
       <c r="R29" s="1"/>
+      <c r="S29" s="1"/>
     </row>
-    <row r="30" spans="1:18" ht="30" x14ac:dyDescent="0.25">
-      <c r="B30" s="12" t="s">
+    <row r="30" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="B30" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C30" s="12" t="s">
+      <c r="C30" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D30" s="12" t="s">
+      <c r="D30" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="E30" s="12" t="s">
+      <c r="E30" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="F30" s="13" t="s">
+      <c r="F30" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="G30" s="13" t="s">
+      <c r="G30" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="H30" s="14" t="s">
+      <c r="H30" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I30" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="J30" s="14"/>
-      <c r="K30" s="1"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18"/>
+      <c r="K30" s="14"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
       <c r="N30" s="1"/>
@@ -31333,8 +32664,9 @@
       <c r="P30" s="1"/>
       <c r="Q30" s="1"/>
       <c r="R30" s="1"/>
+      <c r="S30" s="1"/>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
         <v>2</v>
       </c>
@@ -31357,17 +32689,18 @@
         <v>51.66</v>
       </c>
       <c r="I31" s="16"/>
-      <c r="J31" s="3"/>
-      <c r="K31" s="1"/>
+      <c r="J31" s="16"/>
+      <c r="K31" s="3"/>
       <c r="L31" s="1"/>
-      <c r="M31" s="3"/>
+      <c r="M31" s="1"/>
       <c r="N31" s="3"/>
       <c r="O31" s="3"/>
-      <c r="P31" s="1"/>
+      <c r="P31" s="3"/>
       <c r="Q31" s="1"/>
       <c r="R31" s="1"/>
+      <c r="S31" s="1"/>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B32" s="1" t="s">
         <v>3</v>
       </c>
@@ -31390,17 +32723,18 @@
         <v>41.27935076</v>
       </c>
       <c r="I32" s="1"/>
-      <c r="J32" s="3"/>
-      <c r="K32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="3"/>
       <c r="L32" s="1"/>
-      <c r="M32" s="3"/>
+      <c r="M32" s="1"/>
       <c r="N32" s="3"/>
       <c r="O32" s="3"/>
-      <c r="P32" s="1"/>
+      <c r="P32" s="3"/>
       <c r="Q32" s="1"/>
       <c r="R32" s="1"/>
+      <c r="S32" s="1"/>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
         <v>4</v>
       </c>
@@ -31422,20 +32756,19 @@
       <c r="H33" s="15">
         <v>6.7843516800000003</v>
       </c>
-      <c r="I33" s="1">
-        <v>9023.75</v>
-      </c>
-      <c r="J33" s="3"/>
-      <c r="K33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="3"/>
       <c r="L33" s="1"/>
-      <c r="M33" s="3"/>
+      <c r="M33" s="1"/>
       <c r="N33" s="3"/>
       <c r="O33" s="3"/>
-      <c r="P33" s="9"/>
-      <c r="Q33" s="1"/>
+      <c r="P33" s="3"/>
+      <c r="Q33" s="9"/>
       <c r="R33" s="1"/>
+      <c r="S33" s="1"/>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B34" s="1" t="s">
         <v>5</v>
       </c>
@@ -31457,19 +32790,18 @@
       <c r="H34" s="15">
         <v>5.3650916630000003</v>
       </c>
-      <c r="I34" s="1">
-        <v>118.5</v>
-      </c>
-      <c r="J34" s="3"/>
-      <c r="L34" s="1"/>
-      <c r="M34" s="3"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="1"/>
+      <c r="K34" s="3"/>
+      <c r="M34" s="1"/>
       <c r="N34" s="3"/>
       <c r="O34" s="3"/>
-      <c r="P34" s="9"/>
-      <c r="Q34" s="1"/>
+      <c r="P34" s="3"/>
+      <c r="Q34" s="9"/>
       <c r="R34" s="1"/>
+      <c r="S34" s="1"/>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>25</v>
       </c>
@@ -31494,20 +32826,19 @@
       <c r="H35" s="15">
         <v>29.943162610000002</v>
       </c>
-      <c r="I35" s="1">
-        <v>2036.95</v>
-      </c>
-      <c r="J35" s="3"/>
-      <c r="K35" s="1"/>
+      <c r="I35" s="1"/>
+      <c r="J35" s="1"/>
+      <c r="K35" s="3"/>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
       <c r="N35" s="1"/>
       <c r="O35" s="1"/>
-      <c r="P35" s="9"/>
-      <c r="Q35" s="1"/>
+      <c r="P35" s="1"/>
+      <c r="Q35" s="9"/>
       <c r="R35" s="1"/>
+      <c r="S35" s="1"/>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B36" s="1" t="s">
         <v>7</v>
       </c>
@@ -31529,20 +32860,19 @@
       <c r="H36" s="15">
         <v>13.904999999999999</v>
       </c>
-      <c r="I36" s="1">
-        <v>2036.95</v>
-      </c>
-      <c r="J36" s="3"/>
-      <c r="K36" s="1"/>
+      <c r="I36" s="1"/>
+      <c r="J36" s="1"/>
+      <c r="K36" s="3"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
       <c r="N36" s="1"/>
       <c r="O36" s="1"/>
-      <c r="P36" s="9"/>
-      <c r="Q36" s="1"/>
+      <c r="P36" s="1"/>
+      <c r="Q36" s="9"/>
       <c r="R36" s="1"/>
+      <c r="S36" s="1"/>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
         <v>17</v>
       </c>
@@ -31558,20 +32888,19 @@
       <c r="H37" s="15">
         <v>7.7779999999999996</v>
       </c>
-      <c r="I37" s="1">
-        <v>365</v>
-      </c>
-      <c r="J37" s="9"/>
-      <c r="K37" s="1"/>
+      <c r="I37" s="1"/>
+      <c r="J37" s="1"/>
+      <c r="K37" s="9"/>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
       <c r="N37" s="1"/>
       <c r="O37" s="1"/>
-      <c r="P37" s="9"/>
-      <c r="Q37" s="1"/>
+      <c r="P37" s="1"/>
+      <c r="Q37" s="9"/>
       <c r="R37" s="1"/>
+      <c r="S37" s="1"/>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>25</v>
       </c>
@@ -31596,20 +32925,19 @@
       <c r="H38" s="15">
         <v>5.5549999999999997</v>
       </c>
-      <c r="I38" s="1">
-        <v>365</v>
-      </c>
-      <c r="J38" s="9"/>
-      <c r="K38" s="1"/>
+      <c r="I38" s="1"/>
+      <c r="J38" s="1"/>
+      <c r="K38" s="9"/>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
       <c r="N38" s="1"/>
       <c r="O38" s="1"/>
-      <c r="P38" s="9"/>
-      <c r="Q38" s="1"/>
+      <c r="P38" s="1"/>
+      <c r="Q38" s="9"/>
       <c r="R38" s="1"/>
+      <c r="S38" s="1"/>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B39" s="1" t="s">
         <v>9</v>
       </c>
@@ -31627,20 +32955,19 @@
       <c r="H39" s="15">
         <v>12.67</v>
       </c>
-      <c r="I39" s="1">
-        <v>351.5</v>
-      </c>
-      <c r="J39" s="9"/>
-      <c r="K39" s="1"/>
+      <c r="I39" s="1"/>
+      <c r="J39" s="1"/>
+      <c r="K39" s="9"/>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
       <c r="N39" s="1"/>
       <c r="O39" s="1"/>
-      <c r="P39" s="9"/>
-      <c r="Q39" s="1"/>
+      <c r="P39" s="1"/>
+      <c r="Q39" s="9"/>
       <c r="R39" s="1"/>
+      <c r="S39" s="1"/>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
         <v>10</v>
       </c>
@@ -31658,20 +32985,19 @@
       <c r="H40" s="15">
         <v>5.3390000000000004</v>
       </c>
-      <c r="I40" s="1">
-        <v>413.75</v>
-      </c>
-      <c r="J40" s="9"/>
-      <c r="K40" s="1"/>
+      <c r="I40" s="1"/>
+      <c r="J40" s="1"/>
+      <c r="K40" s="9"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
       <c r="N40" s="1"/>
       <c r="O40" s="1"/>
-      <c r="P40" s="9"/>
-      <c r="Q40" s="1"/>
+      <c r="P40" s="1"/>
+      <c r="Q40" s="9"/>
       <c r="R40" s="1"/>
+      <c r="S40" s="1"/>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B41" s="1" t="s">
         <v>11</v>
       </c>
@@ -31689,20 +33015,19 @@
       <c r="H41" s="15">
         <v>5.1369999999999996</v>
       </c>
-      <c r="I41" s="1">
-        <v>413.75</v>
-      </c>
-      <c r="J41" s="9"/>
-      <c r="K41" s="1"/>
+      <c r="I41" s="1"/>
+      <c r="J41" s="1"/>
+      <c r="K41" s="9"/>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
-      <c r="P41" s="9"/>
-      <c r="Q41" s="1"/>
+      <c r="P41" s="1"/>
+      <c r="Q41" s="9"/>
       <c r="R41" s="1"/>
+      <c r="S41" s="1"/>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
@@ -31720,8 +33045,9 @@
       <c r="P42" s="1"/>
       <c r="Q42" s="1"/>
       <c r="R42" s="1"/>
+      <c r="S42" s="1"/>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B43" s="1" t="s">
         <v>19</v>
       </c>
@@ -31743,27 +33069,28 @@
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
       <c r="J43" s="1"/>
-      <c r="L43" s="1" t="s">
+      <c r="K43" s="1"/>
+      <c r="M43" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="M43" s="1" t="s">
+      <c r="N43" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="N43" s="1" t="s">
+      <c r="O43" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="O43" s="1" t="s">
+      <c r="P43" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="P43" s="1" t="s">
+      <c r="Q43" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="Q43" s="1" t="s">
+      <c r="R43" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="R43" s="1"/>
+      <c r="S43" s="1"/>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B44" s="1" t="s">
         <v>2</v>
       </c>
@@ -31785,27 +33112,28 @@
       <c r="H44" s="3"/>
       <c r="I44" s="3"/>
       <c r="J44" s="3"/>
-      <c r="L44" s="1" t="s">
+      <c r="K44" s="3"/>
+      <c r="M44" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="M44" s="8">
+      <c r="N44" s="8">
         <v>0.46925034971041901</v>
       </c>
-      <c r="N44" s="8">
+      <c r="O44" s="8">
         <v>-0.57047580585715596</v>
       </c>
-      <c r="O44" s="8">
+      <c r="P44" s="8">
         <v>-0.62489073949006502</v>
       </c>
-      <c r="P44" s="8">
+      <c r="Q44" s="8">
         <v>-0.505884156285488</v>
       </c>
-      <c r="Q44" s="8">
+      <c r="R44" s="8">
         <v>-0.62313135244567197</v>
       </c>
-      <c r="R44" s="1"/>
+      <c r="S44" s="1"/>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B45" s="1" t="s">
         <v>3</v>
       </c>
@@ -31827,27 +33155,28 @@
       <c r="H45" s="3"/>
       <c r="I45" s="3"/>
       <c r="J45" s="3"/>
-      <c r="L45" s="1" t="s">
+      <c r="K45" s="3"/>
+      <c r="M45" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="M45" s="8">
+      <c r="N45" s="8">
         <v>0.52770506265369399</v>
       </c>
-      <c r="N45" s="8">
+      <c r="O45" s="8">
         <v>-0.57441925876348399</v>
       </c>
-      <c r="O45" s="8">
+      <c r="P45" s="8">
         <v>-0.61127875482433702</v>
       </c>
-      <c r="P45" s="8">
+      <c r="Q45" s="8">
         <v>-0.50988466103239405</v>
       </c>
-      <c r="Q45" s="8">
+      <c r="R45" s="8">
         <v>-0.59410954788831905</v>
       </c>
-      <c r="R45" s="1"/>
+      <c r="S45" s="1"/>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B46" s="1" t="s">
         <v>4</v>
       </c>
@@ -31869,28 +33198,29 @@
       <c r="H46" s="3"/>
       <c r="I46" s="3"/>
       <c r="J46" s="3"/>
-      <c r="K46" s="9"/>
-      <c r="L46" s="1" t="s">
+      <c r="K46" s="3"/>
+      <c r="L46" s="9"/>
+      <c r="M46" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="M46" s="8">
+      <c r="N46" s="8">
         <v>0.76151296818251002</v>
       </c>
-      <c r="N46" s="8">
+      <c r="O46" s="8">
         <v>-0.82455849900808098</v>
       </c>
-      <c r="O46" s="8">
+      <c r="P46" s="8">
         <v>-0.53010922957415696</v>
       </c>
-      <c r="P46" s="8">
+      <c r="Q46" s="8">
         <v>-0.67807302432253402</v>
       </c>
-      <c r="Q46" s="8">
+      <c r="R46" s="8">
         <v>-0.81917889363282403</v>
       </c>
-      <c r="R46" s="1"/>
+      <c r="S46" s="1"/>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B47" s="1" t="s">
         <v>5</v>
       </c>
@@ -31912,28 +33242,29 @@
       <c r="H47" s="3"/>
       <c r="I47" s="3"/>
       <c r="J47" s="3"/>
-      <c r="K47" s="9"/>
-      <c r="L47" s="1" t="s">
+      <c r="K47" s="3"/>
+      <c r="L47" s="9"/>
+      <c r="M47" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="M47" s="8">
+      <c r="N47" s="8">
         <v>0.63241662033349</v>
       </c>
-      <c r="N47" s="8">
+      <c r="O47" s="8">
         <v>-0.77305412456000899</v>
       </c>
-      <c r="O47" s="8">
+      <c r="P47" s="8">
         <v>-0.511670862423525</v>
       </c>
-      <c r="P47" s="8">
+      <c r="Q47" s="8">
         <v>-0.62213976025652196</v>
       </c>
-      <c r="Q47" s="8">
+      <c r="R47" s="8">
         <v>-0.76662036881149098</v>
       </c>
-      <c r="R47" s="1"/>
+      <c r="S47" s="1"/>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B48" s="1" t="s">
         <v>6</v>
       </c>
@@ -31955,28 +33286,29 @@
       <c r="H48" s="3"/>
       <c r="I48" s="3"/>
       <c r="J48" s="3"/>
-      <c r="K48" s="9"/>
-      <c r="L48" s="1" t="s">
+      <c r="K48" s="3"/>
+      <c r="L48" s="9"/>
+      <c r="M48" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="M48" s="8">
+      <c r="N48" s="8">
         <v>0.68587815994758305</v>
       </c>
-      <c r="N48" s="8">
+      <c r="O48" s="8">
         <v>-0.74314055155585101</v>
       </c>
-      <c r="O48" s="8">
+      <c r="P48" s="8">
         <v>-0.22155858359451899</v>
       </c>
-      <c r="P48" s="8">
+      <c r="Q48" s="8">
         <v>-0.51680913320449795</v>
       </c>
-      <c r="Q48" s="8">
+      <c r="R48" s="8">
         <v>-0.79093223163479298</v>
       </c>
-      <c r="R48" s="1"/>
+      <c r="S48" s="1"/>
     </row>
-    <row r="49" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B49" s="1" t="s">
         <v>7</v>
       </c>
@@ -31998,28 +33330,29 @@
       <c r="H49" s="3"/>
       <c r="I49" s="3"/>
       <c r="J49" s="3"/>
-      <c r="K49" s="9"/>
-      <c r="L49" s="1" t="s">
+      <c r="K49" s="3"/>
+      <c r="L49" s="9"/>
+      <c r="M49" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="M49" s="8">
+      <c r="N49" s="8">
         <v>0.64478493475432996</v>
       </c>
-      <c r="N49" s="8">
+      <c r="O49" s="8">
         <v>-0.64445784381595494</v>
       </c>
-      <c r="O49" s="8">
+      <c r="P49" s="8">
         <v>-0.24334139198969101</v>
       </c>
-      <c r="P49" s="8">
+      <c r="Q49" s="8">
         <v>-0.34407999236201098</v>
       </c>
-      <c r="Q49" s="8">
+      <c r="R49" s="8">
         <v>-0.52379920048275397</v>
       </c>
-      <c r="R49" s="1"/>
+      <c r="S49" s="1"/>
     </row>
-    <row r="50" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B50" s="1" t="s">
         <v>17</v>
       </c>
@@ -32041,27 +33374,28 @@
       <c r="H50" s="3"/>
       <c r="I50" s="3"/>
       <c r="J50" s="3"/>
-      <c r="L50" s="1" t="s">
+      <c r="K50" s="3"/>
+      <c r="M50" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="M50" s="7">
+      <c r="N50" s="7">
         <v>1.04151195285145</v>
       </c>
-      <c r="N50" s="8">
+      <c r="O50" s="8">
         <v>-0.120988015114778</v>
       </c>
-      <c r="O50" s="7">
+      <c r="P50" s="7">
         <v>9.6450074853088597E-2</v>
       </c>
-      <c r="P50" s="8">
+      <c r="Q50" s="8">
         <v>-5.48657708396144E-2</v>
       </c>
-      <c r="Q50" s="8">
+      <c r="R50" s="8">
         <v>-0.16320255139754999</v>
       </c>
-      <c r="R50" s="1"/>
+      <c r="S50" s="1"/>
     </row>
-    <row r="51" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B51" s="1" t="s">
         <v>18</v>
       </c>
@@ -32083,27 +33417,28 @@
       <c r="H51" s="3"/>
       <c r="I51" s="3"/>
       <c r="J51" s="3"/>
-      <c r="L51" s="1" t="s">
+      <c r="K51" s="3"/>
+      <c r="M51" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="M51" s="8">
+      <c r="N51" s="8">
         <v>0.57916197400143898</v>
       </c>
-      <c r="N51" s="8">
+      <c r="O51" s="8">
         <v>-0.78477741945709301</v>
       </c>
-      <c r="O51" s="8">
+      <c r="P51" s="8">
         <v>-0.24313716774511701</v>
       </c>
-      <c r="P51" s="8">
+      <c r="Q51" s="8">
         <v>-0.62437814022779903</v>
       </c>
-      <c r="Q51" s="8">
+      <c r="R51" s="8">
         <v>-0.748656600612842</v>
       </c>
-      <c r="R51" s="1"/>
+      <c r="S51" s="1"/>
     </row>
-    <row r="52" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B52" s="1" t="s">
         <v>11</v>
       </c>
@@ -32125,28 +33460,29 @@
       <c r="H52" s="3"/>
       <c r="I52" s="3"/>
       <c r="J52" s="3"/>
-      <c r="K52" s="9"/>
-      <c r="L52" s="1" t="s">
+      <c r="K52" s="3"/>
+      <c r="L52" s="9"/>
+      <c r="M52" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M52" s="8">
+      <c r="N52" s="8">
         <v>0.74506131022172795</v>
       </c>
-      <c r="N52" s="8">
+      <c r="O52" s="8">
         <v>-0.75894808346496501</v>
       </c>
-      <c r="O52" s="8">
+      <c r="P52" s="8">
         <v>-0.37958282657101999</v>
       </c>
-      <c r="P52" s="8">
+      <c r="Q52" s="8">
         <v>-0.37092334927613402</v>
       </c>
-      <c r="Q52" s="8">
+      <c r="R52" s="8">
         <v>-0.49092006249230202</v>
       </c>
-      <c r="R52" s="1"/>
+      <c r="S52" s="1"/>
     </row>
-    <row r="53" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
       <c r="D53" s="1"/>
@@ -32164,6 +33500,7 @@
       <c r="P53" s="1"/>
       <c r="Q53" s="1"/>
       <c r="R53" s="1"/>
+      <c r="S53" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>